<commit_message>
progress on using salinity for MAD
</commit_message>
<xml_diff>
--- a/spreadsheets/501-all-water-data_Master_23_03.xlsx
+++ b/spreadsheets/501-all-water-data_Master_23_03.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e255fabf6a46c9b0/Desktop/Work stuff/SURF 2026/MAD-FF-Corrections-from-Varied-Salinity/spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{5141D5E6-0ADA-46C2-8933-C0360E65B71F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13A184E9-24FF-485E-ABA4-54F9CBD44D0E}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{5141D5E6-0ADA-46C2-8933-C0360E65B71F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EBEB33E-1493-466E-9559-609043464367}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Interstitial water" sheetId="1" r:id="rId1"/>
@@ -4247,6 +4247,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>